<commit_message>
feat: Generate NBA prediction results, implement data caching, and update debug HTML.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-24.xlsx
+++ b/results/nba_predictions_2025-12-24.xlsx
@@ -568,10 +568,10 @@
         <v>44.83</v>
       </c>
       <c r="F2" t="n">
-        <v>55.38</v>
+        <v>55.31</v>
       </c>
       <c r="G2" t="n">
-        <v>44.62</v>
+        <v>44.69</v>
       </c>
       <c r="H2" t="n">
         <v>-0.1</v>
@@ -614,7 +614,7 @@
         <v>44.8</v>
       </c>
       <c r="T2" t="n">
-        <v>51.9</v>
+        <v>59.6</v>
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
@@ -645,10 +645,10 @@
         <v>32.14</v>
       </c>
       <c r="F3" t="n">
-        <v>58.98</v>
+        <v>59.04</v>
       </c>
       <c r="G3" t="n">
-        <v>41.02</v>
+        <v>40.96</v>
       </c>
       <c r="H3" t="n">
         <v>0.66</v>
@@ -691,7 +691,7 @@
         <v>32.1</v>
       </c>
       <c r="T3" t="n">
-        <v>32.5</v>
+        <v>73.8</v>
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
@@ -722,10 +722,10 @@
         <v>41.67</v>
       </c>
       <c r="F4" t="n">
-        <v>58.48</v>
+        <v>58.46</v>
       </c>
       <c r="G4" t="n">
-        <v>41.52</v>
+        <v>41.54</v>
       </c>
       <c r="H4" t="n">
         <v>0.24</v>
@@ -768,7 +768,7 @@
         <v>41.7</v>
       </c>
       <c r="T4" t="n">
-        <v>39.3</v>
+        <v>88</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
@@ -799,10 +799,10 @@
         <v>60.38</v>
       </c>
       <c r="F5" t="n">
-        <v>53.44</v>
+        <v>53.47</v>
       </c>
       <c r="G5" t="n">
-        <v>46.56</v>
+        <v>46.53</v>
       </c>
       <c r="H5" t="n">
         <v>-0.26</v>
@@ -845,7 +845,7 @@
         <v>60.4</v>
       </c>
       <c r="T5" t="n">
-        <v>59.9</v>
+        <v>79.5</v>
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
@@ -876,10 +876,10 @@
         <v>60.38</v>
       </c>
       <c r="F6" t="n">
-        <v>58.66</v>
+        <v>58.69</v>
       </c>
       <c r="G6" t="n">
-        <v>41.34</v>
+        <v>41.31</v>
       </c>
       <c r="H6" t="n">
         <v>-0.06</v>
@@ -922,7 +922,7 @@
         <v>60.4</v>
       </c>
       <c r="T6" t="n">
-        <v>20.4</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>

</xml_diff>